<commit_message>
min, max, mean spike delay cmputed and plotted for each mfc
</commit_message>
<xml_diff>
--- a/Spike_delay_days.xlsx
+++ b/Spike_delay_days.xlsx
@@ -480,379 +480,377 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.3399305555555556</v>
+        <v>0.339931</v>
       </c>
       <c r="B2" t="n">
-        <v>0.3263888888888889</v>
+        <v>0.326389</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2934027777777778</v>
+        <v>0.293403</v>
       </c>
       <c r="D2" t="n">
-        <v>1.155902777777778</v>
+        <v>1.155903</v>
       </c>
       <c r="E2" t="n">
-        <v>1.167361111111111</v>
+        <v>1.167361</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4243055555555555</v>
+        <v>0.424306</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3572916666666667</v>
+        <v>0.357292</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2364583333333333</v>
+        <v>0.236458</v>
       </c>
       <c r="I2" t="n">
         <v>0.21875</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2930555555555556</v>
+        <v>0.293056</v>
       </c>
       <c r="K2" t="n">
-        <v>0.3270833333333333</v>
+        <v>0.327083</v>
       </c>
       <c r="L2" t="n">
-        <v>0.2694444444444444</v>
+        <v>0.269444</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.1850694444444445</v>
+        <v>0.185069</v>
       </c>
       <c r="B3" t="n">
         <v>0.19375</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2326388888888889</v>
+        <v>0.232639</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2815972222222222</v>
+        <v>0.281597</v>
       </c>
       <c r="E3" t="n">
-        <v>0.001736111111111111</v>
+        <v>0.001736</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2493055555555556</v>
+        <v>0.249306</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1659722222222222</v>
+        <v>0.165972</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1604166666666667</v>
+        <v>0.160417</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1815972222222222</v>
+        <v>0.181597</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1920138888888889</v>
+        <v>0.192014</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.166667</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1607638888888889</v>
+        <v>0.160764</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.2732638888888889</v>
+        <v>0.273264</v>
       </c>
       <c r="B4" t="n">
-        <v>0.3090277777777778</v>
+        <v>0.309028</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2663194444444444</v>
+        <v>0.266319</v>
       </c>
       <c r="D4" t="n">
         <v>0.284375</v>
       </c>
       <c r="E4" t="n">
-        <v>3.999895833333333</v>
+        <v>3.969444</v>
       </c>
       <c r="F4" t="n">
-        <v>2.269444444444444</v>
+        <v>2.269444</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1482638888888889</v>
+        <v>0.148264</v>
       </c>
       <c r="H4" t="n">
-        <v>0.05104166666666667</v>
+        <v>0.051042</v>
       </c>
       <c r="I4" t="n">
         <v>0.19375</v>
       </c>
       <c r="J4" t="n">
-        <v>0.2104166666666667</v>
+        <v>0.210417</v>
       </c>
       <c r="K4" t="n">
-        <v>0.2045138888888889</v>
+        <v>0.204514</v>
       </c>
       <c r="L4" t="n">
-        <v>0.2020833333333333</v>
+        <v>0.202083</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.3020833333333333</v>
+        <v>0.302083</v>
       </c>
       <c r="B5" t="n">
-        <v>0.3340277777777778</v>
+        <v>0.334028</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2993055555555555</v>
+        <v>0.299306</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0006944444444444445</v>
+        <v>0.000694</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0006944444444444445</v>
+        <v>0.000694</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0003472222222222222</v>
+        <v>0.000347</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.4996527777777778</v>
-      </c>
+        <v>0.000347</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>0.09270833333333334</v>
+        <v>0.092708</v>
       </c>
       <c r="J5" t="n">
-        <v>0.05729166666666666</v>
+        <v>0.057292</v>
       </c>
       <c r="K5" t="n">
         <v>0.1</v>
       </c>
       <c r="L5" t="n">
-        <v>0.08541666666666667</v>
+        <v>0.08541700000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.3548611111111111</v>
+        <v>0.354861</v>
       </c>
       <c r="B6" t="n">
-        <v>0.3385416666666667</v>
+        <v>0.338542</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3597222222222222</v>
+        <v>0.359722</v>
       </c>
       <c r="D6" t="n">
-        <v>0.5309027777777777</v>
+        <v>0.530903</v>
       </c>
       <c r="E6" t="n">
-        <v>1.026041666666667</v>
+        <v>1.026042</v>
       </c>
       <c r="F6" t="n">
-        <v>0.5111111111111111</v>
+        <v>0.511111</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5836805555555555</v>
+        <v>0.583681</v>
       </c>
       <c r="H6" t="n">
-        <v>0.04583333333333333</v>
+        <v>0.499653</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2902777777777778</v>
+        <v>0.290278</v>
       </c>
       <c r="J6" t="n">
-        <v>0.4850694444444444</v>
+        <v>0.485069</v>
       </c>
       <c r="K6" t="n">
         <v>0.459375</v>
       </c>
       <c r="L6" t="n">
-        <v>0.4458333333333334</v>
+        <v>0.445833</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.6149305555555555</v>
+        <v>0.614931</v>
       </c>
       <c r="B7" t="n">
         <v>0.6375</v>
       </c>
       <c r="C7" t="n">
-        <v>0.7170138888888888</v>
+        <v>0.717014</v>
       </c>
       <c r="D7" t="n">
-        <v>1.056597222222222</v>
+        <v>1.056597</v>
       </c>
       <c r="E7" t="n">
-        <v>1.037152777777778</v>
+        <v>1.037153</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5642361111111112</v>
+        <v>0.564236</v>
       </c>
       <c r="G7" t="n">
-        <v>0.08055555555555556</v>
+        <v>0.080556</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1006944444444444</v>
+        <v>0.045833</v>
       </c>
       <c r="I7" t="n">
-        <v>0.04756944444444444</v>
+        <v>0.047569</v>
       </c>
       <c r="J7" t="n">
-        <v>0.06180555555555556</v>
+        <v>0.061806</v>
       </c>
       <c r="K7" t="n">
-        <v>0.08784722222222222</v>
+        <v>0.08784699999999999</v>
       </c>
       <c r="L7" t="n">
-        <v>0.2336805555555556</v>
+        <v>0.233681</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.166667</v>
       </c>
       <c r="B8" t="n">
-        <v>0.2638888888888889</v>
+        <v>0.263889</v>
       </c>
       <c r="C8" t="n">
         <v>0.4375</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.111111</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3506944444444444</v>
+        <v>0.350694</v>
       </c>
       <c r="F8" t="n">
-        <v>0.2881944444444444</v>
+        <v>0.288194</v>
       </c>
       <c r="G8" t="n">
-        <v>2.038194444444445</v>
+        <v>2.038194</v>
       </c>
       <c r="H8" t="n">
-        <v>0.4829861111111111</v>
+        <v>0.100694</v>
       </c>
       <c r="I8" t="n">
-        <v>0.1527777777777778</v>
+        <v>0.152778</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>0.003472</v>
       </c>
       <c r="K8" t="n">
         <v>0.15625</v>
       </c>
       <c r="L8" t="n">
-        <v>8.078703703703704</v>
+        <v>8.052083</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.4604166666666666</v>
+        <v>0.460417</v>
       </c>
       <c r="B9" t="n">
-        <v>0.4059027777777778</v>
+        <v>0.405903</v>
       </c>
       <c r="C9" t="n">
-        <v>0.5229166666666667</v>
+        <v>0.522917</v>
       </c>
       <c r="D9" t="n">
         <v>1.05625</v>
       </c>
       <c r="E9" t="n">
-        <v>1.008680555555556</v>
+        <v>1.008681</v>
       </c>
       <c r="F9" t="n">
-        <v>0.6520833333333333</v>
+        <v>0.652083</v>
       </c>
       <c r="G9" t="n">
         <v>0.584375</v>
       </c>
       <c r="H9" t="n">
-        <v>0.08437500000000001</v>
+        <v>0.482986</v>
       </c>
       <c r="I9" t="n">
-        <v>0.4451388888888889</v>
+        <v>0.445139</v>
       </c>
       <c r="J9" t="n">
-        <v>0.3288194444444444</v>
+        <v>0.328819</v>
       </c>
       <c r="K9" t="n">
-        <v>0.5503472222222222</v>
+        <v>0.550347</v>
       </c>
       <c r="L9" t="n">
-        <v>0.5229166666666667</v>
+        <v>0.522917</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.3354166666666666</v>
+        <v>0.335417</v>
       </c>
       <c r="B10" t="n">
-        <v>0.4541666666666667</v>
+        <v>0.454167</v>
       </c>
       <c r="C10" t="n">
-        <v>0.4076388888888889</v>
+        <v>0.407639</v>
       </c>
       <c r="D10" t="n">
-        <v>0.5118055555555555</v>
+        <v>0.511806</v>
       </c>
       <c r="E10" t="n">
-        <v>0.3392361111111111</v>
+        <v>0.339236</v>
       </c>
       <c r="F10" t="n">
         <v>0.590625</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2145833333333333</v>
+        <v>0.214583</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1256944444444444</v>
+        <v>0.08437500000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1270833333333333</v>
+        <v>0.127083</v>
       </c>
       <c r="J10" t="n">
-        <v>0.2197916666666667</v>
+        <v>0.219792</v>
       </c>
       <c r="K10" t="n">
         <v>0.13125</v>
       </c>
       <c r="L10" t="n">
-        <v>0.2260416666666667</v>
+        <v>0.226042</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.3975694444444444</v>
+        <v>0.397569</v>
       </c>
       <c r="B11" t="n">
-        <v>0.3243055555555556</v>
+        <v>0.324306</v>
       </c>
       <c r="C11" t="n">
-        <v>0.3069444444444445</v>
+        <v>0.306944</v>
       </c>
       <c r="D11" t="n">
-        <v>0.3694444444444445</v>
+        <v>0.369444</v>
       </c>
       <c r="E11" t="n">
-        <v>0.2246527777777778</v>
+        <v>0.224653</v>
       </c>
       <c r="F11" t="n">
-        <v>0.4173611111111111</v>
+        <v>0.417361</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1708333333333333</v>
+        <v>0.170833</v>
       </c>
       <c r="H11" t="n">
-        <v>0.3694444444444445</v>
+        <v>0.125694</v>
       </c>
       <c r="I11" t="n">
-        <v>0.1246527777777778</v>
+        <v>0.124653</v>
       </c>
       <c r="J11" t="n">
-        <v>0.09756944444444444</v>
+        <v>0.097569</v>
       </c>
       <c r="K11" t="n">
-        <v>0.09513888888888888</v>
+        <v>0.095139</v>
       </c>
       <c r="L11" t="n">
         <v>0.121875</v>
@@ -860,154 +858,152 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.5159722222222223</v>
+        <v>0.515972</v>
       </c>
       <c r="B12" t="n">
-        <v>0.4371527777777778</v>
+        <v>0.437153</v>
       </c>
       <c r="C12" t="n">
-        <v>3.505902777777778</v>
+        <v>3.505903</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1336805555555556</v>
+        <v>0.133681</v>
       </c>
       <c r="E12" t="n">
         <v>0.33125</v>
       </c>
       <c r="F12" t="n">
-        <v>1.338194444444444</v>
+        <v>1.338194</v>
       </c>
       <c r="G12" t="n">
-        <v>0.3767361111111111</v>
+        <v>0.376736</v>
       </c>
       <c r="H12" t="n">
-        <v>0.7034722222222223</v>
+        <v>0.369444</v>
       </c>
       <c r="I12" t="n">
-        <v>0.1951388888888889</v>
+        <v>0.195139</v>
       </c>
       <c r="J12" t="n">
-        <v>0.3621527777777778</v>
+        <v>0.362153</v>
       </c>
       <c r="K12" t="n">
-        <v>3.130902777777778</v>
+        <v>3.130903</v>
       </c>
       <c r="L12" t="n">
-        <v>0.2684027777777778</v>
+        <v>0.268403</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.4888888888888889</v>
+        <v>0.488889</v>
       </c>
       <c r="B13" t="n">
-        <v>0.5479166666666667</v>
+        <v>0.547917</v>
       </c>
       <c r="C13" t="n">
         <v>0.940625</v>
       </c>
       <c r="D13" t="n">
-        <v>0.6319444444444444</v>
+        <v>0.631944</v>
       </c>
       <c r="E13" t="n">
-        <v>0.5708333333333333</v>
+        <v>0.570833</v>
       </c>
       <c r="F13" t="n">
-        <v>0.7579861111111111</v>
+        <v>0.757986</v>
       </c>
       <c r="G13" t="n">
-        <v>1.353819444444444</v>
+        <v>1.353819</v>
       </c>
       <c r="H13" t="n">
-        <v>1.9125</v>
+        <v>0.703472</v>
       </c>
       <c r="I13" t="n">
-        <v>0.5003472222222223</v>
+        <v>0.500347</v>
       </c>
       <c r="J13" t="n">
-        <v>0.5635416666666667</v>
+        <v>0.563542</v>
       </c>
       <c r="K13" t="n">
-        <v>0.4295138888888889</v>
+        <v>0.429514</v>
       </c>
       <c r="L13" t="n">
-        <v>16.67395833333333</v>
+        <v>16.673958</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1.381944444444444</v>
+        <v>1.381944</v>
       </c>
       <c r="B14" t="n">
-        <v>1.553472222222222</v>
+        <v>1.553472</v>
       </c>
       <c r="C14" t="n">
-        <v>1.487152777777778</v>
+        <v>1.487153</v>
       </c>
       <c r="D14" t="n">
-        <v>59.00579861111111</v>
+        <v>1.094444</v>
       </c>
       <c r="E14" t="n">
-        <v>59.00892361111111</v>
+        <v>1.148958</v>
       </c>
       <c r="F14" t="n">
-        <v>59.00336805555555</v>
+        <v>1.16875</v>
       </c>
       <c r="G14" t="n">
         <v>3.01875</v>
       </c>
       <c r="H14" t="n">
-        <v>0.06076388888888889</v>
+        <v>1.9125</v>
       </c>
       <c r="I14" t="n">
-        <v>1.104166666666667</v>
+        <v>1.104167</v>
       </c>
       <c r="J14" t="n">
-        <v>59.00059027777777</v>
+        <v>0.9246529999999999</v>
       </c>
       <c r="K14" t="n">
-        <v>59.00996527777778</v>
+        <v>1.176736</v>
       </c>
       <c r="L14" t="n">
-        <v>1.120833333333333</v>
+        <v>1.120833</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.2861111111111111</v>
+        <v>0.286111</v>
       </c>
       <c r="B15" t="n">
-        <v>0.2961805555555556</v>
+        <v>0.296181</v>
       </c>
       <c r="C15" t="n">
-        <v>0.2895833333333334</v>
+        <v>0.289583</v>
       </c>
       <c r="D15" t="n">
-        <v>2.988194444444444</v>
+        <v>0.756944</v>
       </c>
       <c r="E15" t="n">
-        <v>2.986805555555556</v>
+        <v>0.000347</v>
       </c>
       <c r="F15" t="n">
-        <v>3.996215277777778</v>
+        <v>1.306944</v>
       </c>
       <c r="G15" t="n">
-        <v>2.986111111111111</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.2052083333333333</v>
-      </c>
+        <v>0.046528</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
         <v>0.34375</v>
       </c>
       <c r="J15" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.133333</v>
       </c>
       <c r="K15" t="n">
-        <v>0.1503472222222222</v>
+        <v>0.150347</v>
       </c>
       <c r="L15" t="n">
-        <v>0.1565972222222222</v>
+        <v>0.156597</v>
       </c>
     </row>
     <row r="16">
@@ -1015,303 +1011,303 @@
         <v>0.396875</v>
       </c>
       <c r="B16" t="n">
-        <v>0.3277777777777778</v>
+        <v>0.327778</v>
       </c>
       <c r="C16" t="n">
-        <v>0.6614583333333334</v>
+        <v>0.661458</v>
       </c>
       <c r="D16" t="n">
         <v>2.21875</v>
       </c>
       <c r="E16" t="n">
-        <v>1.124652777777778</v>
+        <v>1.124653</v>
       </c>
       <c r="F16" t="n">
-        <v>0.9708333333333333</v>
+        <v>0.9708329999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0763888888888889</v>
+        <v>0.076389</v>
       </c>
       <c r="H16" t="n">
-        <v>0.07395833333333333</v>
+        <v>0.060764</v>
       </c>
       <c r="I16" t="n">
-        <v>0.07256944444444445</v>
+        <v>0.07256899999999999</v>
       </c>
       <c r="J16" t="n">
-        <v>0.1545138888888889</v>
+        <v>0.154514</v>
       </c>
       <c r="K16" t="n">
-        <v>1.317361111111111</v>
+        <v>1.317361</v>
       </c>
       <c r="L16" t="n">
-        <v>0.1329861111111111</v>
+        <v>0.132986</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.2701388888888889</v>
+        <v>0.270139</v>
       </c>
       <c r="B17" t="n">
-        <v>0.2576388888888889</v>
+        <v>0.257639</v>
       </c>
       <c r="C17" t="n">
-        <v>0.3302083333333333</v>
+        <v>0.330208</v>
       </c>
       <c r="D17" t="n">
-        <v>0.4059027777777778</v>
+        <v>0.405903</v>
       </c>
       <c r="E17" t="n">
-        <v>0.1010416666666667</v>
+        <v>0.101042</v>
       </c>
       <c r="F17" t="n">
-        <v>0.2513888888888889</v>
+        <v>0.251389</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1305555555555556</v>
+        <v>0.130556</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1003472222222222</v>
+        <v>0.205208</v>
       </c>
       <c r="I17" t="n">
-        <v>0.1006944444444444</v>
+        <v>0.100694</v>
       </c>
       <c r="J17" t="n">
-        <v>0.1444444444444444</v>
+        <v>0.144444</v>
       </c>
       <c r="K17" t="n">
-        <v>0.1743055555555555</v>
+        <v>0.174306</v>
       </c>
       <c r="L17" t="n">
-        <v>0.1986111111111111</v>
+        <v>0.198611</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.1378472222222222</v>
+        <v>0.137847</v>
       </c>
       <c r="B18" t="n">
-        <v>0.2388888888888889</v>
+        <v>0.238889</v>
       </c>
       <c r="C18" t="n">
-        <v>0.2100694444444444</v>
+        <v>0.210069</v>
       </c>
       <c r="D18" t="n">
-        <v>0.1413194444444444</v>
+        <v>0.141319</v>
       </c>
       <c r="E18" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.555556</v>
       </c>
       <c r="F18" t="n">
-        <v>0.4746527777777778</v>
+        <v>0.474653</v>
       </c>
       <c r="G18" t="n">
-        <v>0.09236111111111112</v>
+        <v>0.092361</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>0.073958</v>
       </c>
       <c r="I18" t="n">
-        <v>0.0642361111111111</v>
+        <v>0.064236</v>
       </c>
       <c r="J18" t="n">
-        <v>0.08854166666666667</v>
+        <v>0.088542</v>
       </c>
       <c r="K18" t="n">
         <v>0.053125</v>
       </c>
       <c r="L18" t="n">
-        <v>0.06145833333333333</v>
+        <v>0.061458</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.2659722222222222</v>
+        <v>0.265972</v>
       </c>
       <c r="B19" t="n">
-        <v>0.4527777777777778</v>
+        <v>0.452778</v>
       </c>
       <c r="C19" t="n">
-        <v>0.2194444444444444</v>
+        <v>0.219444</v>
       </c>
       <c r="D19" t="n">
-        <v>0.4454861111111111</v>
+        <v>0.445486</v>
       </c>
       <c r="E19" t="n">
-        <v>0.04479166666666667</v>
+        <v>0.044792</v>
       </c>
       <c r="F19" t="n">
-        <v>0.2715277777777778</v>
+        <v>0.271528</v>
       </c>
       <c r="G19" t="n">
-        <v>0.0920138888888889</v>
+        <v>0.092014</v>
       </c>
       <c r="H19" t="n">
-        <v>0.1694444444444445</v>
+        <v>0.100347</v>
       </c>
       <c r="I19" t="n">
         <v>0.1</v>
       </c>
       <c r="J19" t="n">
-        <v>0.09305555555555556</v>
+        <v>0.093056</v>
       </c>
       <c r="K19" t="n">
-        <v>0.05243055555555556</v>
+        <v>0.052431</v>
       </c>
       <c r="L19" t="n">
-        <v>0.06770833333333333</v>
+        <v>0.067708</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.0006944444444444445</v>
+        <v>0.000694</v>
       </c>
       <c r="B20" t="n">
-        <v>0.0006944444444444445</v>
+        <v>0.000694</v>
       </c>
       <c r="C20" t="n">
-        <v>0.0006944444444444445</v>
+        <v>0.000694</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>0.000347</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>0.000347</v>
       </c>
       <c r="F20" t="n">
-        <v>0.005902777777777778</v>
+        <v>0.005903</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>0.000347</v>
       </c>
       <c r="H20" t="n">
-        <v>0.02118055555555556</v>
+        <v>0.000347</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>0.000347</v>
       </c>
       <c r="J20" t="n">
-        <v>0.4913194444444444</v>
+        <v>0.491319</v>
       </c>
       <c r="K20" t="n">
-        <v>0.02673611111111111</v>
+        <v>0.026736</v>
       </c>
       <c r="L20" t="n">
-        <v>0.0003472222222222222</v>
+        <v>0.000347</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.1972222222222222</v>
+        <v>0.197222</v>
       </c>
       <c r="B21" t="n">
-        <v>0.1979166666666667</v>
+        <v>0.197917</v>
       </c>
       <c r="C21" t="n">
-        <v>0.2510416666666667</v>
+        <v>0.251042</v>
       </c>
       <c r="D21" t="n">
-        <v>0.3034722222222222</v>
+        <v>0.303472</v>
       </c>
       <c r="E21" t="n">
-        <v>0.1392361111111111</v>
+        <v>0.139236</v>
       </c>
       <c r="F21" t="n">
-        <v>0.2211805555555555</v>
+        <v>0.221181</v>
       </c>
       <c r="G21" t="n">
         <v>0.146875</v>
       </c>
       <c r="H21" t="n">
-        <v>0.02222222222222222</v>
+        <v>0.169444</v>
       </c>
       <c r="I21" t="n">
         <v>0.08749999999999999</v>
       </c>
       <c r="J21" t="n">
-        <v>0.1010416666666667</v>
+        <v>0.101042</v>
       </c>
       <c r="K21" t="n">
-        <v>0.1267361111111111</v>
+        <v>0.126736</v>
       </c>
       <c r="L21" t="n">
-        <v>0.03402777777777777</v>
+        <v>0.034028</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0.3197916666666666</v>
+        <v>0.319792</v>
       </c>
       <c r="B22" t="n">
-        <v>0.4395833333333333</v>
+        <v>0.439583</v>
       </c>
       <c r="C22" t="n">
-        <v>0.4697916666666667</v>
+        <v>0.469792</v>
       </c>
       <c r="D22" t="n">
-        <v>0.5826388888888889</v>
+        <v>0.582639</v>
       </c>
       <c r="E22" t="n">
         <v>0.5375</v>
       </c>
       <c r="F22" t="n">
-        <v>0.4722222222222222</v>
+        <v>0.472222</v>
       </c>
       <c r="G22" t="n">
-        <v>0.05243055555555556</v>
+        <v>0.052431</v>
       </c>
       <c r="H22" t="n">
-        <v>0.01736111111111111</v>
+        <v>0.021181</v>
       </c>
       <c r="I22" t="n">
-        <v>0.07395833333333333</v>
+        <v>0.073958</v>
       </c>
       <c r="J22" t="n">
-        <v>0.1184027777777778</v>
+        <v>0.118403</v>
       </c>
       <c r="K22" t="n">
-        <v>0.1649305555555556</v>
+        <v>0.164931</v>
       </c>
       <c r="L22" t="n">
-        <v>0.2385416666666667</v>
+        <v>0.238542</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0.02881944444444445</v>
+        <v>0.028819</v>
       </c>
       <c r="B23" t="n">
-        <v>0.1631944444444444</v>
+        <v>0.163194</v>
       </c>
       <c r="C23" t="n">
-        <v>0.2107638888888889</v>
+        <v>0.210764</v>
       </c>
       <c r="D23" t="n">
-        <v>0.8059027777777777</v>
+        <v>0.805903</v>
       </c>
       <c r="E23" t="n">
-        <v>0.7958333333333333</v>
+        <v>0.795833</v>
       </c>
       <c r="F23" t="n">
-        <v>0.7881944444444444</v>
+        <v>0.788194</v>
       </c>
       <c r="G23" t="n">
-        <v>0.03368055555555555</v>
+        <v>0.033681</v>
       </c>
       <c r="H23" t="n">
-        <v>0.0920138888888889</v>
+        <v>0.022222</v>
       </c>
       <c r="I23" t="n">
-        <v>0.1177083333333333</v>
+        <v>0.117708</v>
       </c>
       <c r="J23" t="n">
-        <v>0.03194444444444444</v>
+        <v>0.031944</v>
       </c>
       <c r="K23" t="n">
-        <v>0.04201388888888889</v>
+        <v>0.042014</v>
       </c>
       <c r="L23" t="n">
-        <v>0.04548611111111111</v>
+        <v>0.045486</v>
       </c>
     </row>
     <row r="24">
@@ -1319,118 +1315,118 @@
         <v>0.190625</v>
       </c>
       <c r="B24" t="n">
-        <v>0.1690972222222222</v>
+        <v>0.169097</v>
       </c>
       <c r="C24" t="n">
-        <v>0.1857638888888889</v>
+        <v>0.185764</v>
       </c>
       <c r="D24" t="n">
-        <v>0.2722222222222222</v>
+        <v>0.272222</v>
       </c>
       <c r="E24" t="n">
-        <v>0.9826388888888888</v>
+        <v>0.982639</v>
       </c>
       <c r="F24" t="n">
         <v>0.21875</v>
       </c>
       <c r="G24" t="n">
-        <v>0.02430555555555556</v>
+        <v>0.024306</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1309027777777778</v>
+        <v>0.017361</v>
       </c>
       <c r="I24" t="n">
         <v>0.09375</v>
       </c>
       <c r="J24" t="n">
-        <v>0.03055555555555555</v>
+        <v>0.030556</v>
       </c>
       <c r="K24" t="n">
-        <v>0.02534722222222222</v>
+        <v>0.025347</v>
       </c>
       <c r="L24" t="n">
-        <v>0.03611111111111111</v>
+        <v>0.036111</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0.1649305555555556</v>
+        <v>0.164931</v>
       </c>
       <c r="B25" t="n">
-        <v>0.1475694444444444</v>
+        <v>0.147569</v>
       </c>
       <c r="C25" t="n">
-        <v>0.1517361111111111</v>
+        <v>0.151736</v>
       </c>
       <c r="D25" t="n">
         <v>0.003125</v>
       </c>
       <c r="E25" t="n">
-        <v>0.1065972222222222</v>
+        <v>0.106597</v>
       </c>
       <c r="F25" t="n">
-        <v>0.4368055555555556</v>
+        <v>0.436806</v>
       </c>
       <c r="G25" t="n">
-        <v>0.04340277777777778</v>
+        <v>0.043403</v>
       </c>
       <c r="H25" t="n">
-        <v>0.01527777777777778</v>
+        <v>0.092014</v>
       </c>
       <c r="I25" t="n">
-        <v>0.05416666666666667</v>
+        <v>0.054167</v>
       </c>
       <c r="J25" t="n">
-        <v>0.08020833333333334</v>
+        <v>0.080208</v>
       </c>
       <c r="K25" t="n">
         <v>0.115625</v>
       </c>
       <c r="L25" t="n">
-        <v>0.1034722222222222</v>
+        <v>0.103472</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>0.001041666666666667</v>
+        <v>0.001042</v>
       </c>
       <c r="B26" t="n">
-        <v>0.1322916666666667</v>
+        <v>0.132292</v>
       </c>
       <c r="C26" t="n">
-        <v>0.1541666666666667</v>
+        <v>0.154167</v>
       </c>
       <c r="D26" t="n">
-        <v>0.001041666666666667</v>
+        <v>0.001042</v>
       </c>
       <c r="E26" t="n">
-        <v>0.001388888888888889</v>
+        <v>0.001389</v>
       </c>
       <c r="F26" t="n">
-        <v>0.1604166666666667</v>
+        <v>0.160417</v>
       </c>
       <c r="G26" t="n">
-        <v>0.08472222222222223</v>
+        <v>0.08472200000000001</v>
       </c>
       <c r="H26" t="n">
-        <v>0.040625</v>
+        <v>0.130903</v>
       </c>
       <c r="I26" t="n">
-        <v>0.1041666666666667</v>
+        <v>0.104167</v>
       </c>
       <c r="J26" t="n">
-        <v>0.07291666666666667</v>
+        <v>0.072917</v>
       </c>
       <c r="K26" t="n">
-        <v>0.08993055555555556</v>
+        <v>0.089931</v>
       </c>
       <c r="L26" t="n">
-        <v>0.1017361111111111</v>
+        <v>0.101736</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>0.2024305555555556</v>
+        <v>0.202431</v>
       </c>
       <c r="B27" t="n">
         <v>0.328125</v>
@@ -1442,102 +1438,104 @@
         <v>0.8375</v>
       </c>
       <c r="E27" t="n">
-        <v>0.8315972222222222</v>
+        <v>0.831597</v>
       </c>
       <c r="F27" t="n">
-        <v>0.5048611111111111</v>
+        <v>0.504861</v>
       </c>
       <c r="G27" t="n">
-        <v>0.07083333333333333</v>
+        <v>0.07083299999999999</v>
       </c>
       <c r="H27" t="n">
-        <v>0.09305555555555556</v>
+        <v>0.015278</v>
       </c>
       <c r="I27" t="n">
-        <v>0.06701388888888889</v>
+        <v>0.067014</v>
       </c>
       <c r="J27" t="n">
-        <v>0.05763888888888889</v>
+        <v>0.057639</v>
       </c>
       <c r="K27" t="n">
-        <v>0.04340277777777778</v>
+        <v>0.043403</v>
       </c>
       <c r="L27" t="n">
-        <v>0.05763888888888889</v>
+        <v>0.057639</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0.05243055555555556</v>
+        <v>0.052431</v>
       </c>
       <c r="B28" t="n">
-        <v>0.0003472222222222222</v>
+        <v>0.000347</v>
       </c>
       <c r="C28" t="n">
-        <v>0.1052083333333333</v>
+        <v>0.105208</v>
       </c>
       <c r="D28" t="n">
-        <v>0.001388888888888889</v>
+        <v>0.001389</v>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>0.000347</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4107638888888889</v>
+        <v>0.410764</v>
       </c>
       <c r="G28" t="n">
-        <v>0.02881944444444445</v>
+        <v>0.028819</v>
       </c>
       <c r="H28" t="n">
-        <v>0.3892361111111111</v>
+        <v>0.040625</v>
       </c>
       <c r="I28" t="n">
-        <v>0.2701388888888889</v>
+        <v>0.270139</v>
       </c>
       <c r="J28" t="n">
-        <v>0.1364583333333333</v>
+        <v>0.136458</v>
       </c>
       <c r="K28" t="n">
-        <v>0.2725694444444444</v>
+        <v>0.272569</v>
       </c>
       <c r="L28" t="n">
-        <v>1.017013888888889</v>
+        <v>1.017014</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>0.1576388888888889</v>
+        <v>0.157639</v>
       </c>
       <c r="B29" t="n">
-        <v>0.1447916666666667</v>
+        <v>0.144792</v>
       </c>
       <c r="C29" t="n">
-        <v>0.1395833333333333</v>
+        <v>0.139583</v>
       </c>
       <c r="D29" t="n">
-        <v>0.2270833333333333</v>
+        <v>0.227083</v>
       </c>
       <c r="E29" t="n">
-        <v>0.2121527777777778</v>
+        <v>0.212153</v>
       </c>
       <c r="F29" t="n">
-        <v>0.3475694444444444</v>
+        <v>0.347569</v>
       </c>
       <c r="G29" t="n">
-        <v>0.09270833333333334</v>
-      </c>
-      <c r="H29" t="inlineStr"/>
+        <v>0.092708</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.093056</v>
+      </c>
       <c r="I29" t="n">
-        <v>0.05833333333333333</v>
+        <v>0.058333</v>
       </c>
       <c r="J29" t="n">
-        <v>0.08819444444444445</v>
+        <v>0.08819399999999999</v>
       </c>
       <c r="K29" t="n">
-        <v>0.07743055555555556</v>
+        <v>0.077431</v>
       </c>
       <c r="L29" t="n">
-        <v>0.1177083333333333</v>
+        <v>0.117708</v>
       </c>
     </row>
     <row r="30">
@@ -1545,7 +1543,7 @@
         <v>0</v>
       </c>
       <c r="B30" t="n">
-        <v>0.2704861111111111</v>
+        <v>0.270486</v>
       </c>
       <c r="C30" t="n">
         <v>0.378125</v>
@@ -1560,20 +1558,22 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>0.4934027777777778</v>
-      </c>
-      <c r="H30" t="inlineStr"/>
+        <v>0.493403</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.389236</v>
+      </c>
       <c r="I30" t="n">
-        <v>0.02673611111111111</v>
+        <v>0.026736</v>
       </c>
       <c r="J30" t="n">
-        <v>0.3204861111111111</v>
+        <v>0.320486</v>
       </c>
       <c r="K30" t="n">
-        <v>0.1298611111111111</v>
+        <v>0.129861</v>
       </c>
       <c r="L30" t="n">
-        <v>0.8635416666666667</v>
+        <v>0.863542</v>
       </c>
     </row>
   </sheetData>

</xml_diff>